<commit_message>
Fix: remove hardcoded credentials, add PUT request, fix duplicate tests, round-trip consistency, real Excel data
</commit_message>
<xml_diff>
--- a/docs/test_documentation.xlsx
+++ b/docs/test_documentation.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
   <si>
     <t>R</t>
   </si>
@@ -104,13 +104,25 @@
     <t>7</t>
   </si>
   <si>
+    <t>PUT</t>
+  </si>
+  <si>
+    <t>Full replacement via PUT (task requirement)</t>
+  </si>
+  <si>
+    <t>Status 200, response has data.id and data.policy_number, response time &lt;2s</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
     <t>Partially update a policy (single field)</t>
   </si>
   <si>
     <t>Status 200, only changed field is updated, data.status changed to cancelled, response time &lt;2s</t>
   </si>
   <si>
-    <t>8</t>
+    <t>9</t>
   </si>
   <si>
     <t>/policies/:policy_id/endorsements</t>
@@ -122,7 +134,7 @@
     <t>Status 201, response has data.id, data.endorsement_type field, response time &lt;2s</t>
   </si>
   <si>
-    <t>9</t>
+    <t>10</t>
   </si>
   <si>
     <t>Retrieve all endorsements for a policy</t>
@@ -131,7 +143,7 @@
     <t>Status 200, response has data array, each endorsement has id field, response time &lt;2s</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>DELETE</t>
@@ -143,7 +155,7 @@
     <t>Status 204, no response body, response time &lt;2s</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
   </si>
   <si>
     <t>/accounts/:id</t>
@@ -167,7 +179,7 @@
     <t>200</t>
   </si>
   <si>
-    <t>{"token":"eyJhbGciOiJIUzI1NiJ9.eyJ1c2VyX2lkIjoiMTJmNzIxMjQtZWI0Yy00MTBmLWEwZTctMDQxYmY4MjJjMjA2IiwiZXhwIjoxNzgxMzI5MDMyLCJpYXQiOjE3ODEyNDI2MzJ9.YOAEOv...</t>
+    <t>{"token":"eyJhbGciOiJIUzI1NiJ9.eyJ1c2VyX2lkIjoiMTJmNzIxMjQtZWI0Yy00MTBmLWEwZTctMDQxYmY4MjJjMjA2IiwiZXhwIjoxNzgxMzMwMDIyLCJpYXQiOjE3ODEyNDM2MjJ9.Y9SJ55...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/auth/login'
@@ -181,7 +193,7 @@
     <t>201</t>
   </si>
   <si>
-    <t>{"data":{"address":{"address_line1":"123 Main St","address_line2":null,"city":"Austin","state":"TX","zip_code":"78701"},"created_at":"2026-06-12T05:37...</t>
+    <t>{"data":{"address":{"address_line1":"123 Main St","address_line2":null,"city":"Austin","state":"TX","zip_code":"78701"},"created_at":"2026-06-12T05:53...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/accounts'
@@ -193,7 +205,7 @@
     <t>Create Policy</t>
   </si>
   <si>
-    <t>{"data":{"account_id":"a967005f-fd80-4e8d-a0ae-b7cf76f4a668","coverage":100000000,"created_at":"2026-06-12T05:37:13.274Z","description":null,"effectiv...</t>
+    <t>{"data":{"account_id":"215737b9-f424-461a-a5ab-5c4da16a07d7","coverage":100000000,"created_at":"2026-06-12T05:53:43.877Z","description":null,"effectiv...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/policies'
@@ -215,7 +227,7 @@
     <t>Get Policy by ID</t>
   </si>
   <si>
-    <t>{"data":{"account":{"email":"alice.1840085094@example.com","first_name":"Alice","id":"a967005f-fd80-4e8d-a0ae-b7cf76f4a668","last_name":"Smith"},"acco...</t>
+    <t>{"data":{"account":{"email":"alice.1328870206@example.com","first_name":"Alice","id":"215737b9-f424-461a-a5ab-5c4da16a07d7","last_name":"Smith"},"acco...</t>
   </si>
   <si>
     <t>curl --location --request GET 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
@@ -225,7 +237,7 @@
     <t>Update Policy (full)</t>
   </si>
   <si>
-    <t>{"data":{"account_id":"a967005f-fd80-4e8d-a0ae-b7cf76f4a668","coverage":200000000,"created_at":"2026-06-12T05:37:13.274Z","description":null,"effectiv...</t>
+    <t>{"data":{"account_id":"215737b9-f424-461a-a5ab-5c4da16a07d7","coverage":200000000,"created_at":"2026-06-12T05:53:43.877Z","description":null,"effectiv...</t>
   </si>
   <si>
     <t>curl --location --request PATCH 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
@@ -236,10 +248,19 @@
     <t>Update Policy (partial)</t>
   </si>
   <si>
+    <t>Update Policy (PUT)</t>
+  </si>
+  <si>
+    <t>curl --location --request PUT 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
+  --header 'Content-Type: application/json'
+  --header 'Authorization: Bearer {{auth_token}}'
+ ...</t>
+  </si>
+  <si>
     <t>Create Endorsement</t>
   </si>
   <si>
-    <t>{"data":{"created_at":"2026-06-12T05:37:15.800Z","description":"Added additional insured rider.","effective_date":"2026-06-12","endorsement_type":"pol...</t>
+    <t>{"data":{"created_at":"2026-06-12T05:53:46.304Z","description":"Added additional insured rider.","effective_date":"2026-06-12","endorsement_type":"pol...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}/endorsements'
@@ -250,7 +271,7 @@
     <t>Get All Endorsements</t>
   </si>
   <si>
-    <t>{"data":[{"created_at":"2026-06-12T05:37:15.800Z","effective_date":"2026-06-12","endorsement_type":"policy_change","id":"9dc962f2-4c5a-4707-974d-c7187...</t>
+    <t>{"data":[{"created_at":"2026-06-12T05:53:46.304Z","effective_date":"2026-06-12","endorsement_type":"policy_change","id":"70c5a703-1a80-4bb5-8528-39302...</t>
   </si>
   <si>
     <t>curl --location --request GET 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}/endorsements'
@@ -486,24 +507,24 @@
         <v>23</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>35</v>
@@ -517,27 +538,27 @@
         <v>37</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>42</v>
@@ -551,16 +572,33 @@
         <v>44</v>
       </c>
       <c r="B16" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="0" t="s">
         <v>45</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>41</v>
       </c>
       <c r="D16" s="0" t="s">
         <v>46</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>43</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -601,7 +639,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -611,15 +649,15 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>7</v>
@@ -628,21 +666,21 @@
         <v>6</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>7</v>
@@ -651,21 +689,21 @@
         <v>11</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>7</v>
@@ -674,21 +712,21 @@
         <v>15</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>19</v>
@@ -697,21 +735,21 @@
         <v>15</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>19</v>
@@ -720,21 +758,21 @@
         <v>23</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>27</v>
@@ -743,21 +781,21 @@
         <v>23</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>27</v>
@@ -766,151 +804,174 @@
         <v>23</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="E15" s="0" t="s">
         <v>55</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>51</v>
+        <v>88</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="E21" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="G20" s="0" t="s">
+      <c r="F21" s="0" t="s">
         <v>89</v>
+      </c>
+      <c r="G21" s="0" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Excel headers: rename Name to Request Name, add Req # column
</commit_message>
<xml_diff>
--- a/docs/test_documentation.xlsx
+++ b/docs/test_documentation.xlsx
@@ -9,21 +9,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>T</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+  <si>
+    <t>Req #</t>
+  </si>
+  <si>
+    <t>Endpoint</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Test Cases / Expected Results</t>
   </si>
   <si>
     <t>1</t>
@@ -164,10 +164,16 @@
     <t>Delete an account</t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>c</t>
+    <t>Request Name</t>
+  </si>
+  <si>
+    <t>Status Code</t>
+  </si>
+  <si>
+    <t>Response Body (Preview)</t>
+  </si>
+  <si>
+    <t>cURL Command</t>
   </si>
   <si>
     <t/>
@@ -179,12 +185,12 @@
     <t>200</t>
   </si>
   <si>
-    <t>{"token":"eyJhbGciOiJIUzI1NiJ9.eyJ1c2VyX2lkIjoiMTJmNzIxMjQtZWI0Yy00MTBmLWEwZTctMDQxYmY4MjJjMjA2IiwiZXhwIjoxNzgxMzMwMDIyLCJpYXQiOjE3ODEyNDM2MjJ9.Y9SJ55...</t>
+    <t>{"token":"eyJhbGciOiJIUzI1NiJ9.eyJ1c2VyX2lkIjoiMTJmNzIxMjQtZWI0Yy00MTBmLWEwZTctMDQxYmY4MjJjMjA2IiwiZXhwIjoxNzgxMzMwNzM3LCJpYXQiOjE3ODEyNDQzMzd9.IB6SXb...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/auth/login'
-  --header 'Content-Type: application/json'
-  --data-raw '{"email":"tskh@gmail.com","password":"Gangsta56"}'</t>
+  --header ''
+  --data-raw '{"email":"{{email}}","password":"{{password}}"}'</t>
   </si>
   <si>
     <t>Create Account</t>
@@ -193,89 +199,97 @@
     <t>201</t>
   </si>
   <si>
-    <t>{"data":{"address":{"address_line1":"123 Main St","address_line2":null,"city":"Austin","state":"TX","zip_code":"78701"},"created_at":"2026-06-12T05:53...</t>
+    <t>{"data":{"address":{"address_line1":"123 Main St","address_line2":null,"city":"Austin","state":"TX","zip_code":"78701"},"created_at":"2026-06-12T06:05...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/accounts'
-  --header 'Content-Type: application/json'
-  --header 'Authorization: Bearer {{auth_token}}'
-  --data-raw '{"accoun...</t>
+  --header ''
+  --header ''
+  --data-raw '{"account":{"first_name":"{{$randomFirstName}}","last_name":"{{$randomLast...</t>
   </si>
   <si>
     <t>Create Policy</t>
   </si>
   <si>
-    <t>{"data":{"account_id":"215737b9-f424-461a-a5ab-5c4da16a07d7","coverage":100000000,"created_at":"2026-06-12T05:53:43.877Z","description":null,"effectiv...</t>
+    <t>{"data":{"account_id":"b6820c7b-7867-4a4d-b895-cd4c6c5d2a15","coverage":100000000,"created_at":"2026-06-12T06:05:37.985Z","description":null,"effectiv...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/policies'
-  --header 'Content-Type: application/json'
-  --header 'Authorization: Bearer {{auth_token}}'
-  --data-raw '{"policy...</t>
+  --header ''
+  --header ''
+  --data-raw '{"policy":{"account_id":"{{created_account_id}}","insurance_type":"general...</t>
   </si>
   <si>
     <t>Get All Policies</t>
   </si>
   <si>
-    <t>{"data":[{"account":{"first_name":"Aliaksandra","id":"ae160337-4d80-40e8-b1e6-1b247033ff4f","last_name":"Pleuskaya"},"account_id":"ae160337-4d80-40e8-...</t>
+    <t>(10052 chars - array of policies)</t>
   </si>
   <si>
     <t>curl --location --request GET 'https://pms.srv1505121.hstgr.cloud/api/v1/policies'
-  --header 'Authorization: Bearer {{auth_token}}'</t>
+  --header ''</t>
   </si>
   <si>
     <t>Get Policy by ID</t>
   </si>
   <si>
-    <t>{"data":{"account":{"email":"alice.1328870206@example.com","first_name":"Alice","id":"215737b9-f424-461a-a5ab-5c4da16a07d7","last_name":"Smith"},"acco...</t>
+    <t>{"data":{"account":{"email":"alice.1710146761@example.com","first_name":"Alice","id":"b6820c7b-7867-4a4d-b895-cd4c6c5d2a15","last_name":"Smith"},"acco...</t>
   </si>
   <si>
     <t>curl --location --request GET 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
-  --header 'Authorization: Bearer {{auth_token}}'</t>
+  --header ''</t>
   </si>
   <si>
     <t>Update Policy (full)</t>
   </si>
   <si>
-    <t>{"data":{"account_id":"215737b9-f424-461a-a5ab-5c4da16a07d7","coverage":200000000,"created_at":"2026-06-12T05:53:43.877Z","description":null,"effectiv...</t>
+    <t>{"data":{"account_id":"b6820c7b-7867-4a4d-b895-cd4c6c5d2a15","coverage":200000000,"created_at":"2026-06-12T06:05:37.985Z","description":null,"effectiv...</t>
   </si>
   <si>
     <t>curl --location --request PATCH 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
-  --header 'Content-Type: application/json'
-  --header 'Authorization: Bearer {{auth_token}}'...</t>
+  --header ''
+  --header ''
+  --data-raw '{"policy":{"insurance_type":"professional_liability...</t>
   </si>
   <si>
     <t>Update Policy (partial)</t>
   </si>
   <si>
+    <t>curl --location --request PATCH 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
+  --header ''
+  --header ''
+  --data-raw '{"policy":{"status":"cancelled"}}'</t>
+  </si>
+  <si>
     <t>Update Policy (PUT)</t>
   </si>
   <si>
     <t>curl --location --request PUT 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
-  --header 'Content-Type: application/json'
-  --header 'Authorization: Bearer {{auth_token}}'
- ...</t>
+  --header ''
+  --header ''
+  --data-raw '{"policy":{"insurance_type":"general_liability","stat...</t>
   </si>
   <si>
     <t>Create Endorsement</t>
   </si>
   <si>
-    <t>{"data":{"created_at":"2026-06-12T05:53:46.304Z","description":"Added additional insured rider.","effective_date":"2026-06-12","endorsement_type":"pol...</t>
+    <t>{"data":{"created_at":"2026-06-12T06:05:39.831Z","description":"Added additional insured rider.","effective_date":"2026-06-12","endorsement_type":"pol...</t>
   </si>
   <si>
     <t>curl --location --request POST 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}/endorsements'
-  --header 'Content-Type: application/json'
-  --header 'Authorization: Bearer {{a...</t>
+  --header ''
+  --header ''
+  --data-raw '{"endorsement":{"endorsement_type":"pol...</t>
   </si>
   <si>
     <t>Get All Endorsements</t>
   </si>
   <si>
-    <t>{"data":[{"created_at":"2026-06-12T05:53:46.304Z","effective_date":"2026-06-12","endorsement_type":"policy_change","id":"70c5a703-1a80-4bb5-8528-39302...</t>
+    <t>{"data":[{"created_at":"2026-06-12T06:05:39.831Z","effective_date":"2026-06-12","endorsement_type":"policy_change","id":"84a19f5e-7791-4fe3-b73f-a020a...</t>
   </si>
   <si>
     <t>curl --location --request GET 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}/endorsements'
-  --header 'Authorization: Bearer {{auth_token}}'</t>
+  --header ''</t>
   </si>
   <si>
     <t>Delete Endorsement</t>
@@ -287,7 +301,11 @@
     <t>404</t>
   </si>
   <si>
-    <t>The remote server returned an error: (404) Not Found.</t>
+    <t>(empty - 204 No Content)</t>
+  </si>
+  <si>
+    <t>curl --location --request DELETE 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}/endorsements/{{created_endorsement_id}}'
+  --header ''</t>
   </si>
   <si>
     <t>Delete Policy</t>
@@ -296,28 +314,25 @@
     <t>204</t>
   </si>
   <si>
-    <t>(empty - 204 No Content)</t>
-  </si>
-  <si>
     <t>curl --location --request DELETE 'https://pms.srv1505121.hstgr.cloud/api/v1/policies/{{created_policy_id}}'
-  --header 'Authorization: Bearer {{auth_token}}'</t>
+  --header ''</t>
   </si>
   <si>
     <t>Get All Accounts</t>
   </si>
   <si>
-    <t>{"data":[{"address":{"address_line1":"Test Street","address_line2":"","city":"Tbilisi","state":"","zip_code":"0159"},"created_at":"2026-05-28T13:26:40...</t>
+    <t>(7245 chars - array of accounts)</t>
   </si>
   <si>
     <t>curl --location --request GET 'https://pms.srv1505121.hstgr.cloud/api/v1/accounts'
-  --header 'Authorization: Bearer {{auth_token}}'</t>
+  --header ''</t>
   </si>
   <si>
     <t>Delete Account</t>
   </si>
   <si>
     <t>curl --location --request DELETE 'https://pms.srv1505121.hstgr.cloud/api/v1/accounts/{{created_account_id}}'
-  --header 'Authorization: Bearer {{auth_token}}'</t>
+  --header ''</t>
   </si>
 </sst>
 </file>
@@ -376,228 +391,220 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>4</v>
+        <v>18</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B12" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="0" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="0" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="E17" s="0" t="s">
         <v>47</v>
       </c>
     </row>
@@ -621,357 +628,345 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>0</v>
+        <v>55</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>55</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>1</v>
+        <v>55</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>0</v>
+        <v>55</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="G16" s="0" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="G17" s="0" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="E18" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="F18" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G18" s="0" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="F19" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="G19" s="0" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" s="0" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="F21" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="G21" s="0" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>